<commit_message>
Add accessibility checker and tabset functionality
- Implement QuartoAxeChecker for accessibility checks using axe-core, with JSON, console, and document reporters.
- Create CSS for syntax highlighting in Quarto documents, defining color variables for various code elements.
- Introduce tabset functionality to maintain state across page loads using localStorage, allowing for grouped tab synchronization.
</commit_message>
<xml_diff>
--- a/input/children-in-cci/data.xlsx
+++ b/input/children-in-cci/data.xlsx
@@ -1,46 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP-MIS\OneDrive\Documents\annual_report_scps\input\children-in-cci\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27F70A4-38F8-473C-A2FD-F1B7BB441FB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="CCI_Count" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Child_Category" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PurviewCCI" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FormalEdRatio" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="VocationalTraining" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CCI_Count" sheetId="1" r:id="rId1"/>
+    <sheet name="Child_Category" sheetId="2" r:id="rId2"/>
+    <sheet name="PurviewCCI" sheetId="3" r:id="rId3"/>
+    <sheet name="FormalEdRatio" sheetId="4" r:id="rId4"/>
+    <sheet name="VocationalTraining" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
   <si>
     <t>District</t>
   </si>
   <si>
-    <t xml:space="preserve">Children Home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Children Home CWSN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observation Home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open Shelter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Special Home/ Place of Safety</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Specialized Adoption Agency</t>
+    <t>Children Home</t>
+  </si>
+  <si>
+    <t>Children Home CWSN</t>
+  </si>
+  <si>
+    <t>Observation Home</t>
+  </si>
+  <si>
+    <t>Open Shelter</t>
+  </si>
+  <si>
+    <t>Special Home/ Place of Safety</t>
+  </si>
+  <si>
+    <t>Specialized Adoption Agency</t>
   </si>
   <si>
     <t>Total</t>
@@ -55,10 +59,10 @@
     <t>Birbhum</t>
   </si>
   <si>
-    <t xml:space="preserve">Koch Bihar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dakshin Dinajpur</t>
+    <t>Koch Bihar</t>
+  </si>
+  <si>
+    <t>Dakshin Dinajpur</t>
   </si>
   <si>
     <t>Darjiling</t>
@@ -91,37 +95,37 @@
     <t>Nadia</t>
   </si>
   <si>
-    <t xml:space="preserve">North 24 Parganas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paschim Barddhaman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pashchim Medinipur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Purba Barddhaman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Purba Medinipur</t>
+    <t>North 24 Parganas</t>
+  </si>
+  <si>
+    <t>Paschim Barddhaman</t>
+  </si>
+  <si>
+    <t>Pashchim Medinipur</t>
+  </si>
+  <si>
+    <t>Purba Barddhaman</t>
+  </si>
+  <si>
+    <t>Purba Medinipur</t>
   </si>
   <si>
     <t>Puruliya</t>
   </si>
   <si>
-    <t xml:space="preserve">South 24 Parganas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uttar Dinajpur</t>
+    <t>South 24 Parganas</t>
+  </si>
+  <si>
+    <t>Uttar Dinajpur</t>
   </si>
   <si>
     <t>Category</t>
   </si>
   <si>
-    <t xml:space="preserve">No. of Children</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non-CWSN CNCP</t>
+    <t>No. of Children</t>
+  </si>
+  <si>
+    <t>Non-CWSN CNCP</t>
   </si>
   <si>
     <t>CWSN</t>
@@ -169,10 +173,16 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11.000000"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
@@ -191,23 +201,23 @@
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="2" borderId="0" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="9" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="9" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -227,12 +237,12 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
-  <mc:AlternateContent>
-    <mc:Choice Requires="c14">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
       <c14:style val="102"/>
     </mc:Choice>
     <mc:Fallback>
@@ -247,7 +257,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike">
+              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -267,9 +277,8 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
-      <c:spPr bwMode="auto">
+      <c:spPr>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -284,7 +293,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike">
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -311,7 +320,7 @@
           <c:dPt>
             <c:idx val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr bwMode="auto">
+            <c:spPr>
               <a:prstGeom prst="rect">
                 <a:avLst/>
               </a:prstGeom>
@@ -352,11 +361,16 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-DE71-4B4C-BFD1-4EEE15DE1AB4}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr bwMode="auto">
+            <c:spPr>
               <a:prstGeom prst="rect">
                 <a:avLst/>
               </a:prstGeom>
@@ -397,11 +411,16 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-DE71-4B4C-BFD1-4EEE15DE1AB4}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
             <c:bubble3D val="0"/>
-            <c:spPr bwMode="auto">
+            <c:spPr>
               <a:prstGeom prst="rect">
                 <a:avLst/>
               </a:prstGeom>
@@ -442,8 +461,49 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-DE71-4B4C-BFD1-4EEE15DE1AB4}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr bwMode="auto">
                 <a:prstGeom prst="rect">
@@ -461,45 +521,19 @@
                 <a:effectLst/>
               </c:spPr>
             </c:leaderLines>
-            <c:showBubbleSize val="0"/>
-            <c:showCatName val="0"/>
-            <c:showLeaderLines val="1"/>
-            <c:showLegendKey val="0"/>
-            <c:showPercent val="1"/>
-            <c:showSerName val="0"/>
-            <c:showVal val="0"/>
-            <c:spPr bwMode="auto">
-              <a:prstGeom prst="rect">
-                <a:avLst/>
-              </a:prstGeom>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+              </c:ext>
+            </c:extLst>
           </c:dLbls>
           <c:cat>
             <c:strRef>
@@ -525,30 +559,35 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>2528</c:v>
+                  <c:v>2164</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1428</c:v>
+                  <c:v>1447</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>192</c:v>
+                  <c:v>145</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-DE71-4B4C-BFD1-4EEE15DE1AB4}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
           <c:showBubbleSize val="0"/>
-          <c:showCatName val="0"/>
           <c:showLeaderLines val="1"/>
-          <c:showLegendKey val="0"/>
-          <c:showPercent val="1"/>
-          <c:showSerName val="0"/>
-          <c:showVal val="0"/>
         </c:dLbls>
         <c:firstSliceAng val="0"/>
       </c:pieChart>
-      <c:spPr bwMode="auto">
+      <c:spPr>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -561,9 +600,8 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
-      <c:spPr bwMode="auto">
+      <c:spPr>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -578,7 +616,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike">
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -599,7 +637,7 @@
     <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr bwMode="auto">
-    <a:xfrm rot="0">
+    <a:xfrm>
       <a:off x="0" y="0"/>
       <a:ext cx="0" cy="0"/>
     </a:xfrm>
@@ -632,7 +670,7 @@
   </c:txPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins l="0.69999999999999996" r="0.69999999999999996" t="0.75" b="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -848,6 +886,7 @@
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
@@ -1227,13 +1266,12 @@
       <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:wall>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
 </cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
-  <xdr:twoCellAnchor editAs="twoCell">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>466724</xdr:colOff>
@@ -1246,14 +1284,20 @@
       <xdr:row>25</xdr:row>
       <xdr:rowOff>152399</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame>
+    <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 1"/>
+        <xdr:cNvPr id="4" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
-      <xdr:xfrm rot="0">
+      <xdr:xfrm>
         <a:off x="0" y="0"/>
         <a:ext cx="0" cy="0"/>
       </xdr:xfrm>
@@ -1268,291 +1312,8 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1775,25 +1536,27 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="20.85546875"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" width="14.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" width="20"/>
-    <col bestFit="1" customWidth="1" min="4" max="4" width="17.42578125"/>
-    <col bestFit="1" customWidth="1" min="5" max="5" width="11.375"/>
-    <col bestFit="1" customWidth="1" min="6" max="6" width="27.28515625"/>
-    <col bestFit="1" customWidth="1" min="7" max="7" width="26.42578125"/>
-    <col bestFit="1" customWidth="1" min="8" max="8" width="5.42578125"/>
-    <col bestFit="1" customWidth="1" min="9" max="16384" width="9.140625"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1819,7 +1582,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1845,7 +1608,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1871,7 +1634,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1897,7 +1660,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1923,7 +1686,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1949,7 +1712,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1975,7 +1738,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -2001,7 +1764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -2027,7 +1790,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2053,7 +1816,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -2079,7 +1842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -2105,7 +1868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -2131,7 +1894,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -2157,7 +1920,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -2183,7 +1946,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -2209,7 +1972,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -2235,7 +1998,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -2261,7 +2024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -2287,7 +2050,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -2313,7 +2076,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -2339,7 +2102,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -2365,7 +2128,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -2391,7 +2154,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -2418,26 +2181,23 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="9"/>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="16.28515625"/>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>31</v>
       </c>
@@ -2445,7 +2205,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -2453,7 +2213,7 @@
         <v>2164</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -2461,7 +2221,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -2470,24 +2230,21 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="9"/>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -2501,7 +2258,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -2515,7 +2272,7 @@
         <v>11001</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -2529,7 +2286,7 @@
         <v>11799</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -2543,7 +2300,7 @@
         <v>13105</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>42</v>
       </c>
@@ -2557,7 +2314,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -2571,7 +2328,7 @@
         <v>11711</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -2585,7 +2342,7 @@
         <v>16475</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>45</v>
       </c>
@@ -2599,7 +2356,7 @@
         <v>18097</v>
       </c>
     </row>
-    <row r="9" ht="15">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -2614,23 +2371,20 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="9"/>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -2638,7 +2392,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -2646,7 +2400,7 @@
         <v>0.50955369980068466</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -2654,7 +2408,7 @@
         <v>0.46290806807288964</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -2662,7 +2416,7 @@
         <v>0.47065990190682927</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>42</v>
       </c>
@@ -2670,7 +2424,7 @@
         <v>0.47789022476016468</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -2678,7 +2432,7 @@
         <v>0.47187937096248245</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -2686,7 +2440,7 @@
         <v>0.54675583741089873</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>45</v>
       </c>
@@ -2694,35 +2448,32 @@
         <v>0.56826199145876555</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>46</v>
       </c>
       <c r="B9" s="2">
-        <v>0.52880000000000005</v>
+        <v>0.57879999999999998</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="7.7109375"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -2730,7 +2481,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -2738,7 +2489,7 @@
         <v>0.42307810567844872</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -2746,7 +2497,7 @@
         <v>0.42742471126864257</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -2754,7 +2505,7 @@
         <v>0.39869396131682211</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>42</v>
       </c>
@@ -2762,7 +2513,7 @@
         <v>0.37921372133676096</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -2770,7 +2521,7 @@
         <v>0.35419074400942852</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -2778,7 +2529,7 @@
         <v>0.37807294431195831</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>45</v>
       </c>
@@ -2786,7 +2537,7 @@
         <v>0.42059486459360856</v>
       </c>
     </row>
-    <row r="9" ht="15">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -2795,9 +2546,7 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Update data and figures in Annual Report Fact Sheet
</commit_message>
<xml_diff>
--- a/input/children-in-cci/data.xlsx
+++ b/input/children-in-cci/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP-MIS\OneDrive\Documents\annual_report_scps\input\children-in-cci\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27F70A4-38F8-473C-A2FD-F1B7BB441FB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D66E5C1-B8F8-44BA-886E-2D6C3F2147BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CCI_Count" sheetId="1" r:id="rId1"/>
@@ -86,6 +86,57 @@
     <t>Kolkata</t>
   </si>
   <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>No. of Children</t>
+  </si>
+  <si>
+    <t>Non-CWSN CNCP</t>
+  </si>
+  <si>
+    <t>CWSN</t>
+  </si>
+  <si>
+    <t>CCL</t>
+  </si>
+  <si>
+    <t>FY</t>
+  </si>
+  <si>
+    <t>Girls</t>
+  </si>
+  <si>
+    <t>Boys</t>
+  </si>
+  <si>
+    <t>2017-18</t>
+  </si>
+  <si>
+    <t>2018-19</t>
+  </si>
+  <si>
+    <t>2019-20</t>
+  </si>
+  <si>
+    <t>2020-21</t>
+  </si>
+  <si>
+    <t>2021-22</t>
+  </si>
+  <si>
+    <t>2022-23</t>
+  </si>
+  <si>
+    <t>2023-24</t>
+  </si>
+  <si>
+    <t>2024-25</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
     <t>Maldah</t>
   </si>
   <si>
@@ -117,57 +168,6 @@
   </si>
   <si>
     <t>Uttar Dinajpur</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>No. of Children</t>
-  </si>
-  <si>
-    <t>Non-CWSN CNCP</t>
-  </si>
-  <si>
-    <t>CWSN</t>
-  </si>
-  <si>
-    <t>CCL</t>
-  </si>
-  <si>
-    <t>FY</t>
-  </si>
-  <si>
-    <t>Girls</t>
-  </si>
-  <si>
-    <t>Boys</t>
-  </si>
-  <si>
-    <t>2017-18</t>
-  </si>
-  <si>
-    <t>2018-19</t>
-  </si>
-  <si>
-    <t>2019-20</t>
-  </si>
-  <si>
-    <t>2020-21</t>
-  </si>
-  <si>
-    <t>2021-22</t>
-  </si>
-  <si>
-    <t>2022-23</t>
-  </si>
-  <si>
-    <t>2023-24</t>
-  </si>
-  <si>
-    <t>2024-25</t>
-  </si>
-  <si>
-    <t>average</t>
   </si>
 </sst>
 </file>
@@ -185,6 +185,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -215,9 +216,9 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -288,26 +289,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -505,7 +486,7 @@
             <c:showBubbleSize val="0"/>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
-              <c:spPr bwMode="auto">
+              <c:spPr>
                 <a:prstGeom prst="rect">
                   <a:avLst/>
                 </a:prstGeom>
@@ -527,10 +508,6 @@
                   <a:prstGeom prst="rect">
                     <a:avLst/>
                   </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
                 </c15:spPr>
               </c:ext>
             </c:extLst>
@@ -636,7 +613,7 @@
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
   </c:chart>
-  <c:spPr bwMode="auto">
+  <c:spPr>
     <a:xfrm>
       <a:off x="0" y="0"/>
       <a:ext cx="0" cy="0"/>
@@ -674,599 +651,6 @@
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
-</file>
-
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
-  <a:schemeClr val="accent6"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent4"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="344">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-  </cs:categoryAxis>
-  <cs:chartArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx2"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="34925" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:legend>
-  <cs:plotArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1600" b="1"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr bwMode="auto">
-      <a:prstGeom prst="rect">
-        <a:avLst/>
-      </a:prstGeom>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1743,7 +1127,7 @@
         <v>14</v>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1761,7 +1145,7 @@
         <v>2</v>
       </c>
       <c r="H8">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1778,7 +1162,7 @@
         <v>2</v>
       </c>
       <c r="E9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -1787,7 +1171,7 @@
         <v>3</v>
       </c>
       <c r="H9">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1862,10 +1246,10 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1882,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -1891,12 +1275,12 @@
         <v>9</v>
       </c>
       <c r="H13">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -1922,7 +1306,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="B15">
         <v>8</v>
@@ -1948,7 +1332,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -1974,13 +1358,13 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="B17">
         <v>7</v>
       </c>
       <c r="C17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17">
         <v>2</v>
@@ -1995,12 +1379,12 @@
         <v>1</v>
       </c>
       <c r="H17">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -2026,7 +1410,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="B19">
         <v>12</v>
@@ -2052,7 +1436,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -2078,7 +1462,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B21">
         <v>4</v>
@@ -2104,7 +1488,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -2130,7 +1514,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="B23">
         <v>6</v>
@@ -2139,7 +1523,7 @@
         <v>4</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2151,12 +1535,12 @@
         <v>1</v>
       </c>
       <c r="H23">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="B24">
         <v>2</v>
@@ -2199,15 +1583,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <v>2164</v>
@@ -2215,7 +1599,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1447</v>
@@ -2223,7 +1607,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>145</v>
@@ -2246,13 +1630,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s">
         <v>7</v>
@@ -2260,7 +1644,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B2">
         <v>5931</v>
@@ -2274,7 +1658,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B3">
         <v>5795</v>
@@ -2288,7 +1672,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B4">
         <v>7346</v>
@@ -2302,7 +1686,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B5">
         <v>5221</v>
@@ -2316,7 +1700,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B6">
         <v>7138</v>
@@ -2330,7 +1714,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B7">
         <v>11131</v>
@@ -2344,7 +1728,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B8">
         <v>12958</v>
@@ -2358,7 +1742,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="B9">
         <v>16168</v>
@@ -2386,15 +1770,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
         <v>36</v>
-      </c>
-      <c r="B1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1">
         <v>0.50955369980068466</v>
@@ -2402,7 +1786,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B3" s="1">
         <v>0.46290806807288964</v>
@@ -2410,7 +1794,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B4" s="1">
         <v>0.47065990190682927</v>
@@ -2418,7 +1802,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B5" s="1">
         <v>0.47789022476016468</v>
@@ -2426,7 +1810,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B6" s="1">
         <v>0.47187937096248245</v>
@@ -2434,7 +1818,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B7" s="1">
         <v>0.54675583741089873</v>
@@ -2442,7 +1826,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1">
         <v>0.56826199145876555</v>
@@ -2450,7 +1834,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2">
         <v>0.57879999999999998</v>
@@ -2475,15 +1859,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
         <v>36</v>
-      </c>
-      <c r="B1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B2" s="3">
         <v>0.42307810567844872</v>
@@ -2491,7 +1875,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B3" s="3">
         <v>0.42742471126864257</v>
@@ -2499,7 +1883,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B4" s="3">
         <v>0.39869396131682211</v>
@@ -2507,7 +1891,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B5" s="3">
         <v>0.37921372133676096</v>
@@ -2515,7 +1899,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B6" s="3">
         <v>0.35419074400942852</v>
@@ -2523,7 +1907,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B7" s="3">
         <v>0.37807294431195831</v>
@@ -2531,7 +1915,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B8" s="3">
         <v>0.42059486459360856</v>
@@ -2539,7 +1923,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="B9" s="4">
         <v>0.4556</v>

</xml_diff>